<commit_message>
:sparkles: feat: update json style so each sheet can be different table
</commit_message>
<xml_diff>
--- a/output/sample.xlsx
+++ b/output/sample.xlsx
@@ -456,7 +456,7 @@
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -467,7 +467,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Name</t>
+          <t>Product Name</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -477,7 +477,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Quantity</t>
+          <t>Stock Quantity</t>
         </is>
       </c>
     </row>
@@ -536,22 +536,22 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>Sale ID</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Name</t>
+          <t>Customer</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Price</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Quantity</t>
+          <t>Sale Date</t>
         </is>
       </c>
     </row>
@@ -561,14 +561,16 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Sale A</t>
+          <t>John Doe</t>
         </is>
       </c>
       <c r="C2" s="4" t="n">
         <v>199500</v>
       </c>
-      <c r="D2" s="5" t="n">
-        <v>10</v>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>2024-02-01</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>